<commit_message>
Phase 5: migrate 23 fund detail pages + terms-and-conditions
- fund-detail template validated on 3 diverse samples (flat/multi/nested-groups)
- Bulk-imported all 23 CIT fund pages (23/23 success): hero + fund description + PDF document links (flat or grouped, all preserved) + disclaimer + columns CTA + form
- goalpath: 35 PDF links across nested fund-series groups, all captured
- terms-and-conditions: long legal doc as default content (30/30 paragraphs), legal template
- normalizeFundPage + normalizeLegalPage guarded transformer additions (no-op on other pages)
- All 23 matrix-cits tile links resolve to imported fund pages; lint clean

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-about-us.report.xlsx
+++ b/tools/importer/reports/import-about-us.report.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="52">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="112" uniqueCount="78">
   <si>
     <t>_reportFile</t>
   </si>
@@ -49,7 +49,7 @@
     <t>success</t>
   </si>
   <si>
-    <t>2026-08-11T15:36:02.082Z</t>
+    <t>2026-08-11T17:20:38.914Z</t>
   </si>
   <si>
     <t>Matrix Trust Company | Broadridge</t>
@@ -118,7 +118,7 @@
     <t>cit-landing</t>
   </si>
   <si>
-    <t>2026-08-11T15:14:01.231Z</t>
+    <t>2026-08-11T17:20:30.835Z</t>
   </si>
   <si>
     <t>Collective Investment Trusts | Broadridge</t>
@@ -127,6 +127,57 @@
     <t>https://www.broadridge.com/cit/</t>
   </si>
   <si>
+    <t>equity-armor-cits.report.json</t>
+  </si>
+  <si>
+    <t>equity-armor-cits</t>
+  </si>
+  <si>
+    <t>fund-detail</t>
+  </si>
+  <si>
+    <t>2026-08-11T17:18:46.137Z</t>
+  </si>
+  <si>
+    <t>Equity Armor CITs | Broadridge</t>
+  </si>
+  <si>
+    <t>https://www.broadridge.com/cit/equity-armor-cits</t>
+  </si>
+  <si>
+    <t>financial-advisers.report.json</t>
+  </si>
+  <si>
+    <t>["hero-banner","columns","columns","form-contact"]</t>
+  </si>
+  <si>
+    <t>financial-advisers</t>
+  </si>
+  <si>
+    <t>2026-08-11T15:43:24.842Z</t>
+  </si>
+  <si>
+    <t>Financial Advisers | Broadridge</t>
+  </si>
+  <si>
+    <t>https://www.broadridge.com/cit/financial-advisers</t>
+  </si>
+  <si>
+    <t>goalpath-portfolios.report.json</t>
+  </si>
+  <si>
+    <t>goalpath-portfolios</t>
+  </si>
+  <si>
+    <t>2026-08-11T17:18:52.682Z</t>
+  </si>
+  <si>
+    <t>GoalPath Portfolios | Broadridge</t>
+  </si>
+  <si>
+    <t>https://www.broadridge.com/cit/goalpath-portfolios</t>
+  </si>
+  <si>
     <t>matrix-cits.report.json</t>
   </si>
   <si>
@@ -145,6 +196,21 @@
     <t>https://www.broadridge.com/cit/matrix-cits</t>
   </si>
   <si>
+    <t>mutual-of-america-stable-value-cit.report.json</t>
+  </si>
+  <si>
+    <t>mutual-of-america-stable-value-cit</t>
+  </si>
+  <si>
+    <t>2026-08-11T17:18:38.889Z</t>
+  </si>
+  <si>
+    <t>Mutual of America Stable Value CIT</t>
+  </si>
+  <si>
+    <t>https://www.broadridge.com/cit/mutual-of-america-stable-value-cit</t>
+  </si>
+  <si>
     <t>tpas-and-record-keepers.report.json</t>
   </si>
   <si>
@@ -158,6 +224,18 @@
   </si>
   <si>
     <t>https://www.broadridge.com/cit/tpas-and-record-keepers</t>
+  </si>
+  <si>
+    <t>cit/about-us.report.json</t>
+  </si>
+  <si>
+    <t>["hero-banner","form-contact","columns"]</t>
+  </si>
+  <si>
+    <t>cit/about-us</t>
+  </si>
+  <si>
+    <t>2026-08-11T16:45:11.260Z</t>
   </si>
   <si>
     <t>cit/matrix-cits.report.json</t>
@@ -555,12 +633,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H9"/>
+  <dimension ref="A1:H14"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="1" width="37" customWidth="1"/>
+    <col min="1" max="1" width="48" customWidth="1"/>
     <col min="2" max="2" width="50" customWidth="1"/>
-    <col min="3" max="3" width="25" customWidth="1"/>
+    <col min="3" max="3" width="36" customWidth="1"/>
     <col min="5" max="5" width="25" customWidth="1"/>
     <col min="6" max="6" width="26" customWidth="1"/>
     <col min="7" max="8" width="50" customWidth="1"/>
@@ -727,7 +805,7 @@
         <v>38</v>
       </c>
       <c r="B7" t="s">
-        <v>21</v>
+        <v>9</v>
       </c>
       <c r="C7" t="s">
         <v>39</v>
@@ -753,36 +831,36 @@
         <v>44</v>
       </c>
       <c r="B8" t="s">
-        <v>9</v>
+        <v>45</v>
       </c>
       <c r="C8" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="D8" t="s">
         <v>11</v>
       </c>
       <c r="E8" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="F8" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="G8" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="H8" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B9" t="s">
-        <v>21</v>
+        <v>9</v>
       </c>
       <c r="C9" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="D9" t="s">
         <v>11</v>
@@ -791,13 +869,143 @@
         <v>40</v>
       </c>
       <c r="F9" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="G9" t="s">
-        <v>42</v>
+        <v>53</v>
       </c>
       <c r="H9" t="s">
-        <v>43</v>
+        <v>54</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>55</v>
+      </c>
+      <c r="B10" t="s">
+        <v>21</v>
+      </c>
+      <c r="C10" t="s">
+        <v>56</v>
+      </c>
+      <c r="D10" t="s">
+        <v>11</v>
+      </c>
+      <c r="E10" t="s">
+        <v>57</v>
+      </c>
+      <c r="F10" t="s">
+        <v>58</v>
+      </c>
+      <c r="G10" t="s">
+        <v>59</v>
+      </c>
+      <c r="H10" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>61</v>
+      </c>
+      <c r="B11" t="s">
+        <v>9</v>
+      </c>
+      <c r="C11" t="s">
+        <v>62</v>
+      </c>
+      <c r="D11" t="s">
+        <v>11</v>
+      </c>
+      <c r="E11" t="s">
+        <v>40</v>
+      </c>
+      <c r="F11" t="s">
+        <v>63</v>
+      </c>
+      <c r="G11" t="s">
+        <v>64</v>
+      </c>
+      <c r="H11" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>66</v>
+      </c>
+      <c r="B12" t="s">
+        <v>9</v>
+      </c>
+      <c r="C12" t="s">
+        <v>67</v>
+      </c>
+      <c r="D12" t="s">
+        <v>11</v>
+      </c>
+      <c r="E12" t="s">
+        <v>67</v>
+      </c>
+      <c r="F12" t="s">
+        <v>68</v>
+      </c>
+      <c r="G12" t="s">
+        <v>69</v>
+      </c>
+      <c r="H12" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>71</v>
+      </c>
+      <c r="B13" t="s">
+        <v>72</v>
+      </c>
+      <c r="C13" t="s">
+        <v>73</v>
+      </c>
+      <c r="D13" t="s">
+        <v>11</v>
+      </c>
+      <c r="E13" t="s">
+        <v>34</v>
+      </c>
+      <c r="F13" t="s">
+        <v>74</v>
+      </c>
+      <c r="G13" t="s">
+        <v>13</v>
+      </c>
+      <c r="H13" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>75</v>
+      </c>
+      <c r="B14" t="s">
+        <v>21</v>
+      </c>
+      <c r="C14" t="s">
+        <v>76</v>
+      </c>
+      <c r="D14" t="s">
+        <v>11</v>
+      </c>
+      <c r="E14" t="s">
+        <v>57</v>
+      </c>
+      <c r="F14" t="s">
+        <v>77</v>
+      </c>
+      <c r="G14" t="s">
+        <v>59</v>
+      </c>
+      <c r="H14" t="s">
+        <v>60</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Phase 6 QA: normalize heading hierarchy (WCAG 1.3.1) across all pages
- Add stack-based heading renumbering to broadridge-cleanup transformer:
  removes level skips (h1->h3, h2->h5 from Divi visual sizing) and keeps
  sibling headings (card grids) at the same level
- Re-imported all 32 pages; QA sweep: 0 heading skips, exactly 1 h1/page,
  content imgs have alt, no javascript:/empty links
- Card/column CSS targets headings generically, so no visual regression

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-about-us.report.xlsx
+++ b/tools/importer/reports/import-about-us.report.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="112" uniqueCount="78">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="333" uniqueCount="196">
   <si>
     <t>_reportFile</t>
   </si>
@@ -34,22 +34,46 @@
     <t>title</t>
   </si>
   <si>
+    <t>type</t>
+  </si>
+  <si>
     <t>url</t>
   </si>
   <si>
+    <t>3edge-asset-management.report.json</t>
+  </si>
+  <si>
+    <t>["hero-banner","columns","form-contact"]</t>
+  </si>
+  <si>
+    <t>3edge-asset-management</t>
+  </si>
+  <si>
+    <t>success</t>
+  </si>
+  <si>
+    <t>fund-detail</t>
+  </si>
+  <si>
+    <t>2026-08-12T05:36:56.477Z</t>
+  </si>
+  <si>
+    <t>3EDGE Asset Management | Broadridge</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>https://www.broadridge.com/cit/3edge-asset-management</t>
+  </si>
+  <si>
     <t>about-us.report.json</t>
   </si>
   <si>
-    <t>["hero-banner","columns","form-contact"]</t>
-  </si>
-  <si>
     <t>about-us</t>
   </si>
   <si>
-    <t>success</t>
-  </si>
-  <si>
-    <t>2026-08-11T17:20:38.914Z</t>
+    <t>2026-08-12T05:42:42.666Z</t>
   </si>
   <si>
     <t>Matrix Trust Company | Broadridge</t>
@@ -64,7 +88,7 @@
     <t>banks-and-trusts</t>
   </si>
   <si>
-    <t>2026-08-11T15:24:05.647Z</t>
+    <t>2026-08-12T05:42:17.067Z</t>
   </si>
   <si>
     <t>Matrix Banks and Trusts | Broadridge</t>
@@ -82,7 +106,7 @@
     <t>broker-dealer-platform</t>
   </si>
   <si>
-    <t>2026-08-11T15:35:51.500Z</t>
+    <t>2026-08-12T05:42:08.883Z</t>
   </si>
   <si>
     <t>Broker-Dealer Platform | Broadridge</t>
@@ -97,7 +121,7 @@
     <t>cit-services</t>
   </si>
   <si>
-    <t>2026-08-11T14:50:33.904Z</t>
+    <t>2026-08-12T05:41:58.902Z</t>
   </si>
   <si>
     <t>Collective Investment Trust Services | Broadridge</t>
@@ -118,7 +142,7 @@
     <t>cit-landing</t>
   </si>
   <si>
-    <t>2026-08-11T17:20:30.835Z</t>
+    <t>2026-08-12T05:41:39.515Z</t>
   </si>
   <si>
     <t>Collective Investment Trusts | Broadridge</t>
@@ -127,16 +151,73 @@
     <t>https://www.broadridge.com/cit/</t>
   </si>
   <si>
+    <t>commerce-core-bond-cit.report.json</t>
+  </si>
+  <si>
+    <t>commerce-core-bond-cit</t>
+  </si>
+  <si>
+    <t>2026-08-12T05:42:10.334Z</t>
+  </si>
+  <si>
+    <t>Commerce Core Bond CIT | Broadridge</t>
+  </si>
+  <si>
+    <t>https://www.broadridge.com/cit/commerce-core-bond-cit</t>
+  </si>
+  <si>
+    <t>donaldson-preservation-fund.report.json</t>
+  </si>
+  <si>
+    <t>donaldson-preservation-fund</t>
+  </si>
+  <si>
+    <t>2026-08-12T05:37:09.117Z</t>
+  </si>
+  <si>
+    <t>Donaldson Preservation Fund | Broadridge</t>
+  </si>
+  <si>
+    <t>https://www.broadridge.com/cit/donaldson-preservation-fund</t>
+  </si>
+  <si>
+    <t>donaldson-rising-dividend-fund.report.json</t>
+  </si>
+  <si>
+    <t>donaldson-rising-dividend-fund</t>
+  </si>
+  <si>
+    <t>2026-08-12T05:37:02.484Z</t>
+  </si>
+  <si>
+    <t>Donaldson Rising Dividend | Broadridge</t>
+  </si>
+  <si>
+    <t>https://www.broadridge.com/cit/donaldson-rising-dividend-fund</t>
+  </si>
+  <si>
+    <t>donaldson-sequoia-fund.report.json</t>
+  </si>
+  <si>
+    <t>donaldson-sequoia-fund</t>
+  </si>
+  <si>
+    <t>2026-08-12T05:42:30.434Z</t>
+  </si>
+  <si>
+    <t>Donaldson Sequoia Fund | Broadridge</t>
+  </si>
+  <si>
+    <t>https://www.broadridge.com/cit/donaldson-sequoia-fund</t>
+  </si>
+  <si>
     <t>equity-armor-cits.report.json</t>
   </si>
   <si>
     <t>equity-armor-cits</t>
   </si>
   <si>
-    <t>fund-detail</t>
-  </si>
-  <si>
-    <t>2026-08-11T17:18:46.137Z</t>
+    <t>2026-08-12T05:41:55.560Z</t>
   </si>
   <si>
     <t>Equity Armor CITs | Broadridge</t>
@@ -154,7 +235,7 @@
     <t>financial-advisers</t>
   </si>
   <si>
-    <t>2026-08-11T15:43:24.842Z</t>
+    <t>2026-08-12T05:42:34.106Z</t>
   </si>
   <si>
     <t>Financial Advisers | Broadridge</t>
@@ -163,13 +244,28 @@
     <t>https://www.broadridge.com/cit/financial-advisers</t>
   </si>
   <si>
+    <t>footer.report.json</t>
+  </si>
+  <si>
+    <t>footer</t>
+  </si>
+  <si>
+    <t>2026-08-12T05:11:54.506Z</t>
+  </si>
+  <si>
+    <t>Footer</t>
+  </si>
+  <si>
+    <t>chrome</t>
+  </si>
+  <si>
     <t>goalpath-portfolios.report.json</t>
   </si>
   <si>
     <t>goalpath-portfolios</t>
   </si>
   <si>
-    <t>2026-08-11T17:18:52.682Z</t>
+    <t>2026-08-12T05:37:21.999Z</t>
   </si>
   <si>
     <t>GoalPath Portfolios | Broadridge</t>
@@ -178,6 +274,48 @@
     <t>https://www.broadridge.com/cit/goalpath-portfolios</t>
   </si>
   <si>
+    <t>highland-capital-management-core-fixed-fund.report.json</t>
+  </si>
+  <si>
+    <t>highland-capital-management-core-fixed-fund</t>
+  </si>
+  <si>
+    <t>2026-08-12T05:36:44.738Z</t>
+  </si>
+  <si>
+    <t>Highland Capital Management: SMID Cap Core Alpha Fund | Broadridge</t>
+  </si>
+  <si>
+    <t>https://www.broadridge.com/cit/highland-capital-management-core-fixed-fund</t>
+  </si>
+  <si>
+    <t>highland-capital-management-smid-cap-core-alpha-fund.report.json</t>
+  </si>
+  <si>
+    <t>highland-capital-management-smid-cap-core-alpha-fund</t>
+  </si>
+  <si>
+    <t>2026-08-12T05:36:37.163Z</t>
+  </si>
+  <si>
+    <t>https://www.broadridge.com/cit/highland-capital-management-smid-cap-core-alpha-fund</t>
+  </si>
+  <si>
+    <t>managed-retirement-funds.report.json</t>
+  </si>
+  <si>
+    <t>managed-retirement-funds</t>
+  </si>
+  <si>
+    <t>2026-08-12T05:37:28.436Z</t>
+  </si>
+  <si>
+    <t>Managed Retirement Funds | Broadridge</t>
+  </si>
+  <si>
+    <t>https://www.broadridge.com/cit/managed-retirement-funds</t>
+  </si>
+  <si>
     <t>matrix-cits.report.json</t>
   </si>
   <si>
@@ -187,7 +325,7 @@
     <t>cit-offerings</t>
   </si>
   <si>
-    <t>2026-08-11T15:14:08.996Z</t>
+    <t>2026-08-12T05:41:48.694Z</t>
   </si>
   <si>
     <t>Matrix Trust Company Collective Investment Trusts | Broadridge</t>
@@ -196,13 +334,43 @@
     <t>https://www.broadridge.com/cit/matrix-cits</t>
   </si>
   <si>
+    <t>matrix-trust-multi-manager-stable-value-fund.report.json</t>
+  </si>
+  <si>
+    <t>matrix-trust-multi-manager-stable-value-fund</t>
+  </si>
+  <si>
+    <t>2026-08-12T05:37:15.545Z</t>
+  </si>
+  <si>
+    <t>Matrix Trust Multi Manager Stable Value Fund | Broadridge</t>
+  </si>
+  <si>
+    <t>https://www.broadridge.com/cit/matrix-trust-multi-manager-stable-value-fund</t>
+  </si>
+  <si>
+    <t>mtc-northern-trust.report.json</t>
+  </si>
+  <si>
+    <t>mtc-northern-trust</t>
+  </si>
+  <si>
+    <t>2026-08-12T05:42:37.637Z</t>
+  </si>
+  <si>
+    <t>MTC Northern Trust Index | Broadridge</t>
+  </si>
+  <si>
+    <t>https://www.broadridge.com/cit/mtc-northern-trust</t>
+  </si>
+  <si>
     <t>mutual-of-america-stable-value-cit.report.json</t>
   </si>
   <si>
     <t>mutual-of-america-stable-value-cit</t>
   </si>
   <si>
-    <t>2026-08-11T17:18:38.889Z</t>
+    <t>2026-08-12T05:41:39.489Z</t>
   </si>
   <si>
     <t>Mutual of America Stable Value CIT</t>
@@ -211,19 +379,205 @@
     <t>https://www.broadridge.com/cit/mutual-of-america-stable-value-cit</t>
   </si>
   <si>
+    <t>nav.report.json</t>
+  </si>
+  <si>
+    <t>nav</t>
+  </si>
+  <si>
+    <t>2026-08-12T05:11:40.494Z</t>
+  </si>
+  <si>
+    <t>Navigation</t>
+  </si>
+  <si>
+    <t>pacific-life-income-horizon-cits.report.json</t>
+  </si>
+  <si>
+    <t>pacific-life-income-horizon-cits</t>
+  </si>
+  <si>
+    <t>2026-08-12T05:41:47.781Z</t>
+  </si>
+  <si>
+    <t>Pacific Life Income Horizon CITs | Broadridge</t>
+  </si>
+  <si>
+    <t>https://www.broadridge.com/cit/pacific-life-income-horizon-cits</t>
+  </si>
+  <si>
+    <t>pacific-ridge-small-cap-value.report.json</t>
+  </si>
+  <si>
+    <t>pacific-ridge-small-cap-value</t>
+  </si>
+  <si>
+    <t>2026-08-12T05:42:03.335Z</t>
+  </si>
+  <si>
+    <t>Pacific Ridge Small Cap Value | Broadridge</t>
+  </si>
+  <si>
+    <t>https://www.broadridge.com/cit/pacific-ridge-small-cap-value</t>
+  </si>
+  <si>
+    <t>retirement-advocate-funds.report.json</t>
+  </si>
+  <si>
+    <t>retirement-advocate-funds</t>
+  </si>
+  <si>
+    <t>2026-08-12T05:37:34.403Z</t>
+  </si>
+  <si>
+    <t>Retirement Advocate Funds | Broadridge</t>
+  </si>
+  <si>
+    <t>https://www.broadridge.com/cit/retirement-advocate-funds</t>
+  </si>
+  <si>
+    <t>starpath-funds.report.json</t>
+  </si>
+  <si>
+    <t>["hero-banner","columns"]</t>
+  </si>
+  <si>
+    <t>starpath-funds</t>
+  </si>
+  <si>
+    <t>2026-08-12T05:37:40.474Z</t>
+  </si>
+  <si>
+    <t>StarPath Funds | Broadridge</t>
+  </si>
+  <si>
+    <t>https://www.broadridge.com/cit/starpath-funds</t>
+  </si>
+  <si>
+    <t>strategic-roadmap-portfolios.report.json</t>
+  </si>
+  <si>
+    <t>strategic-roadmap-portfolios</t>
+  </si>
+  <si>
+    <t>2026-08-12T05:37:48.206Z</t>
+  </si>
+  <si>
+    <t>Strategic Roadmap Portfolios | Broadridge</t>
+  </si>
+  <si>
+    <t>https://www.broadridge.com/cit/strategic-roadmap-portfolios</t>
+  </si>
+  <si>
+    <t>terms-and-conditions.report.json</t>
+  </si>
+  <si>
+    <t>["hero-banner"]</t>
+  </si>
+  <si>
+    <t>terms-and-conditions</t>
+  </si>
+  <si>
+    <t>legal</t>
+  </si>
+  <si>
+    <t>2026-08-12T05:32:50.455Z</t>
+  </si>
+  <si>
+    <t>Matrix Terms of Service</t>
+  </si>
+  <si>
+    <t>https://www.broadridge.com/cit/terms-and-conditions</t>
+  </si>
+  <si>
     <t>tpas-and-record-keepers.report.json</t>
   </si>
   <si>
     <t>tpas-and-record-keepers</t>
   </si>
   <si>
-    <t>2026-08-11T15:34:16.431Z</t>
+    <t>2026-08-12T05:42:24.952Z</t>
   </si>
   <si>
     <t>TPAs and Recordkeepers | Broadridge</t>
   </si>
   <si>
     <t>https://www.broadridge.com/cit/tpas-and-record-keepers</t>
+  </si>
+  <si>
+    <t>twelve-points-retirement-advisors-100-percent-equity-fund.report.json</t>
+  </si>
+  <si>
+    <t>twelve-points-retirement-advisors-100-percent-equity-fund</t>
+  </si>
+  <si>
+    <t>2026-08-12T05:36:24.138Z</t>
+  </si>
+  <si>
+    <t>Twelve Points Retirement Advisors 100% Equity Fund | Broadridge</t>
+  </si>
+  <si>
+    <t>https://www.broadridge.com/cit/twelve-points-retirement-advisors-100-percent-equity-fund</t>
+  </si>
+  <si>
+    <t>twelve-points-target-risk-portfolios.report.json</t>
+  </si>
+  <si>
+    <t>twelve-points-target-risk-portfolios</t>
+  </si>
+  <si>
+    <t>2026-08-12T05:36:30.775Z</t>
+  </si>
+  <si>
+    <t>Twelve Points Target Risk Portfolios | Broadridge</t>
+  </si>
+  <si>
+    <t>https://www.broadridge.com/cit/twelve-points-target-risk-portfolios</t>
+  </si>
+  <si>
+    <t>wealthplan-partners-dividend-aristocrats-portfolio-fund.report.json</t>
+  </si>
+  <si>
+    <t>wealthplan-partners-dividend-aristocrats-portfolio-fund</t>
+  </si>
+  <si>
+    <t>2026-08-12T05:36:50.243Z</t>
+  </si>
+  <si>
+    <t>WealthPlan Partners Dividend Aristocrats Portfolio Fund | Broadridge</t>
+  </si>
+  <si>
+    <t>https://www.broadridge.com/cit/wealthplan-partners-dividend-aristocrats-portfolio-fund</t>
+  </si>
+  <si>
+    <t>xponance-inc-small-cap-core-equity-smid-cap-core-equity-funds.report.json</t>
+  </si>
+  <si>
+    <t>xponance-inc-small-cap-core-equity-smid-cap-core-equity-funds</t>
+  </si>
+  <si>
+    <t>2026-08-12T05:42:23.559Z</t>
+  </si>
+  <si>
+    <t>Xponance Inc. Small Cap Core Equity/SMID Cap Core Equity Funds | Broadridge</t>
+  </si>
+  <si>
+    <t>https://www.broadridge.com/cit/xponance-inc-small-cap-core-equity-smid-cap-core-equity-funds</t>
+  </si>
+  <si>
+    <t>xponance-inc-yield-advantage-opportunistic-core-bond-fund.report.json</t>
+  </si>
+  <si>
+    <t>xponance-inc-yield-advantage-opportunistic-core-bond-fund</t>
+  </si>
+  <si>
+    <t>2026-08-12T05:42:16.932Z</t>
+  </si>
+  <si>
+    <t>Xponance Inc. Yield Advantage Opportunistic Core Bond Fund | Broadridge</t>
+  </si>
+  <si>
+    <t>https://www.broadridge.com/cit/xponance-inc-yield-advantage-opportunistic-core-bond-fund</t>
   </si>
   <si>
     <t>cit/about-us.report.json</t>
@@ -633,18 +987,18 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H14"/>
+  <dimension ref="A1:I37"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="1" width="48" customWidth="1"/>
-    <col min="2" max="2" width="50" customWidth="1"/>
-    <col min="3" max="3" width="36" customWidth="1"/>
+    <col min="1" max="3" width="50" customWidth="1"/>
     <col min="5" max="5" width="25" customWidth="1"/>
     <col min="6" max="6" width="26" customWidth="1"/>
-    <col min="7" max="8" width="50" customWidth="1"/>
+    <col min="7" max="7" width="50" customWidth="1"/>
+    <col min="8" max="8" width="8" customWidth="1"/>
+    <col min="9" max="9" width="50" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -669,230 +1023,257 @@
       <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I1" s="1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B2" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C2" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D2" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E2" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="F2" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="G2" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="H2" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+        <v>16</v>
+      </c>
+      <c r="I2" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="B3" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C3" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="D3" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E3" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="F3" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="G3" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="H3" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+        <v>16</v>
+      </c>
+      <c r="I3" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="B4" t="s">
-        <v>21</v>
+        <v>10</v>
       </c>
       <c r="C4" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="D4" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E4" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="F4" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="G4" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="H4" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+        <v>16</v>
+      </c>
+      <c r="I4" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="B5" t="s">
-        <v>9</v>
+        <v>29</v>
       </c>
       <c r="C5" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="D5" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E5" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="F5" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="G5" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="H5" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+        <v>16</v>
+      </c>
+      <c r="I5" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="B6" t="s">
-        <v>32</v>
+        <v>10</v>
       </c>
       <c r="C6" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="D6" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E6" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="F6" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="G6" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="H6" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+        <v>16</v>
+      </c>
+      <c r="I6" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B7" t="s">
-        <v>9</v>
+        <v>40</v>
       </c>
       <c r="C7" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="D7" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E7" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="F7" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="G7" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="H7" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+        <v>16</v>
+      </c>
+      <c r="I7" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="B8" t="s">
-        <v>45</v>
+        <v>10</v>
       </c>
       <c r="C8" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="D8" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E8" t="s">
-        <v>46</v>
+        <v>13</v>
       </c>
       <c r="F8" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="G8" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="H8" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+        <v>16</v>
+      </c>
+      <c r="I8" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B9" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C9" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="D9" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E9" t="s">
-        <v>40</v>
+        <v>13</v>
       </c>
       <c r="F9" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="G9" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="H9" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+        <v>16</v>
+      </c>
+      <c r="I9" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B10" t="s">
-        <v>21</v>
+        <v>10</v>
       </c>
       <c r="C10" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D10" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E10" t="s">
-        <v>57</v>
+        <v>13</v>
       </c>
       <c r="F10" t="s">
         <v>58</v>
@@ -901,24 +1282,27 @@
         <v>59</v>
       </c>
       <c r="H10" t="s">
+        <v>16</v>
+      </c>
+      <c r="I10" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>61</v>
       </c>
       <c r="B11" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C11" t="s">
         <v>62</v>
       </c>
       <c r="D11" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E11" t="s">
-        <v>40</v>
+        <v>13</v>
       </c>
       <c r="F11" t="s">
         <v>63</v>
@@ -927,24 +1311,27 @@
         <v>64</v>
       </c>
       <c r="H11" t="s">
+        <v>16</v>
+      </c>
+      <c r="I11" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>66</v>
       </c>
       <c r="B12" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C12" t="s">
         <v>67</v>
       </c>
       <c r="D12" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E12" t="s">
-        <v>67</v>
+        <v>13</v>
       </c>
       <c r="F12" t="s">
         <v>68</v>
@@ -953,10 +1340,13 @@
         <v>69</v>
       </c>
       <c r="H12" t="s">
+        <v>16</v>
+      </c>
+      <c r="I12" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>71</v>
       </c>
@@ -967,49 +1357,722 @@
         <v>73</v>
       </c>
       <c r="D13" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E13" t="s">
-        <v>34</v>
+        <v>73</v>
       </c>
       <c r="F13" t="s">
         <v>74</v>
       </c>
       <c r="G13" t="s">
-        <v>13</v>
+        <v>75</v>
       </c>
       <c r="H13" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
+        <v>16</v>
+      </c>
+      <c r="I13" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="B14" t="s">
+        <v>16</v>
+      </c>
+      <c r="C14" t="s">
+        <v>78</v>
+      </c>
+      <c r="D14" t="s">
+        <v>12</v>
+      </c>
+      <c r="E14" t="s">
+        <v>16</v>
+      </c>
+      <c r="F14" t="s">
+        <v>79</v>
+      </c>
+      <c r="G14" t="s">
+        <v>80</v>
+      </c>
+      <c r="H14" t="s">
+        <v>81</v>
+      </c>
+      <c r="I14" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>82</v>
+      </c>
+      <c r="B15" t="s">
+        <v>10</v>
+      </c>
+      <c r="C15" t="s">
+        <v>83</v>
+      </c>
+      <c r="D15" t="s">
+        <v>12</v>
+      </c>
+      <c r="E15" t="s">
+        <v>13</v>
+      </c>
+      <c r="F15" t="s">
+        <v>84</v>
+      </c>
+      <c r="G15" t="s">
+        <v>85</v>
+      </c>
+      <c r="H15" t="s">
+        <v>16</v>
+      </c>
+      <c r="I15" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>87</v>
+      </c>
+      <c r="B16" t="s">
+        <v>10</v>
+      </c>
+      <c r="C16" t="s">
+        <v>88</v>
+      </c>
+      <c r="D16" t="s">
+        <v>12</v>
+      </c>
+      <c r="E16" t="s">
+        <v>13</v>
+      </c>
+      <c r="F16" t="s">
+        <v>89</v>
+      </c>
+      <c r="G16" t="s">
+        <v>90</v>
+      </c>
+      <c r="H16" t="s">
+        <v>16</v>
+      </c>
+      <c r="I16" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>92</v>
+      </c>
+      <c r="B17" t="s">
+        <v>10</v>
+      </c>
+      <c r="C17" t="s">
+        <v>93</v>
+      </c>
+      <c r="D17" t="s">
+        <v>12</v>
+      </c>
+      <c r="E17" t="s">
+        <v>13</v>
+      </c>
+      <c r="F17" t="s">
+        <v>94</v>
+      </c>
+      <c r="G17" t="s">
+        <v>90</v>
+      </c>
+      <c r="H17" t="s">
+        <v>16</v>
+      </c>
+      <c r="I17" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>96</v>
+      </c>
+      <c r="B18" t="s">
+        <v>10</v>
+      </c>
+      <c r="C18" t="s">
+        <v>97</v>
+      </c>
+      <c r="D18" t="s">
+        <v>12</v>
+      </c>
+      <c r="E18" t="s">
+        <v>13</v>
+      </c>
+      <c r="F18" t="s">
+        <v>98</v>
+      </c>
+      <c r="G18" t="s">
+        <v>99</v>
+      </c>
+      <c r="H18" t="s">
+        <v>16</v>
+      </c>
+      <c r="I18" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>101</v>
+      </c>
+      <c r="B19" t="s">
+        <v>29</v>
+      </c>
+      <c r="C19" t="s">
+        <v>102</v>
+      </c>
+      <c r="D19" t="s">
+        <v>12</v>
+      </c>
+      <c r="E19" t="s">
+        <v>103</v>
+      </c>
+      <c r="F19" t="s">
+        <v>104</v>
+      </c>
+      <c r="G19" t="s">
+        <v>105</v>
+      </c>
+      <c r="H19" t="s">
+        <v>16</v>
+      </c>
+      <c r="I19" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>107</v>
+      </c>
+      <c r="B20" t="s">
+        <v>10</v>
+      </c>
+      <c r="C20" t="s">
+        <v>108</v>
+      </c>
+      <c r="D20" t="s">
+        <v>12</v>
+      </c>
+      <c r="E20" t="s">
+        <v>13</v>
+      </c>
+      <c r="F20" t="s">
+        <v>109</v>
+      </c>
+      <c r="G20" t="s">
+        <v>110</v>
+      </c>
+      <c r="H20" t="s">
+        <v>16</v>
+      </c>
+      <c r="I20" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>112</v>
+      </c>
+      <c r="B21" t="s">
+        <v>10</v>
+      </c>
+      <c r="C21" t="s">
+        <v>113</v>
+      </c>
+      <c r="D21" t="s">
+        <v>12</v>
+      </c>
+      <c r="E21" t="s">
+        <v>13</v>
+      </c>
+      <c r="F21" t="s">
+        <v>114</v>
+      </c>
+      <c r="G21" t="s">
+        <v>115</v>
+      </c>
+      <c r="H21" t="s">
+        <v>16</v>
+      </c>
+      <c r="I21" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>117</v>
+      </c>
+      <c r="B22" t="s">
+        <v>10</v>
+      </c>
+      <c r="C22" t="s">
+        <v>118</v>
+      </c>
+      <c r="D22" t="s">
+        <v>12</v>
+      </c>
+      <c r="E22" t="s">
+        <v>13</v>
+      </c>
+      <c r="F22" t="s">
+        <v>119</v>
+      </c>
+      <c r="G22" t="s">
+        <v>120</v>
+      </c>
+      <c r="H22" t="s">
+        <v>16</v>
+      </c>
+      <c r="I22" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="23" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>122</v>
+      </c>
+      <c r="B23" t="s">
+        <v>16</v>
+      </c>
+      <c r="C23" t="s">
+        <v>123</v>
+      </c>
+      <c r="D23" t="s">
+        <v>12</v>
+      </c>
+      <c r="E23" t="s">
+        <v>16</v>
+      </c>
+      <c r="F23" t="s">
+        <v>124</v>
+      </c>
+      <c r="G23" t="s">
+        <v>125</v>
+      </c>
+      <c r="H23" t="s">
+        <v>81</v>
+      </c>
+      <c r="I23" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="24" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>126</v>
+      </c>
+      <c r="B24" t="s">
+        <v>10</v>
+      </c>
+      <c r="C24" t="s">
+        <v>127</v>
+      </c>
+      <c r="D24" t="s">
+        <v>12</v>
+      </c>
+      <c r="E24" t="s">
+        <v>13</v>
+      </c>
+      <c r="F24" t="s">
+        <v>128</v>
+      </c>
+      <c r="G24" t="s">
+        <v>129</v>
+      </c>
+      <c r="H24" t="s">
+        <v>16</v>
+      </c>
+      <c r="I24" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="25" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>131</v>
+      </c>
+      <c r="B25" t="s">
+        <v>10</v>
+      </c>
+      <c r="C25" t="s">
+        <v>132</v>
+      </c>
+      <c r="D25" t="s">
+        <v>12</v>
+      </c>
+      <c r="E25" t="s">
+        <v>13</v>
+      </c>
+      <c r="F25" t="s">
+        <v>133</v>
+      </c>
+      <c r="G25" t="s">
+        <v>134</v>
+      </c>
+      <c r="H25" t="s">
+        <v>16</v>
+      </c>
+      <c r="I25" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="26" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>136</v>
+      </c>
+      <c r="B26" t="s">
+        <v>10</v>
+      </c>
+      <c r="C26" t="s">
+        <v>137</v>
+      </c>
+      <c r="D26" t="s">
+        <v>12</v>
+      </c>
+      <c r="E26" t="s">
+        <v>13</v>
+      </c>
+      <c r="F26" t="s">
+        <v>138</v>
+      </c>
+      <c r="G26" t="s">
+        <v>139</v>
+      </c>
+      <c r="H26" t="s">
+        <v>16</v>
+      </c>
+      <c r="I26" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="27" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>141</v>
+      </c>
+      <c r="B27" t="s">
+        <v>142</v>
+      </c>
+      <c r="C27" t="s">
+        <v>143</v>
+      </c>
+      <c r="D27" t="s">
+        <v>12</v>
+      </c>
+      <c r="E27" t="s">
+        <v>13</v>
+      </c>
+      <c r="F27" t="s">
+        <v>144</v>
+      </c>
+      <c r="G27" t="s">
+        <v>145</v>
+      </c>
+      <c r="H27" t="s">
+        <v>16</v>
+      </c>
+      <c r="I27" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="28" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>147</v>
+      </c>
+      <c r="B28" t="s">
+        <v>10</v>
+      </c>
+      <c r="C28" t="s">
+        <v>148</v>
+      </c>
+      <c r="D28" t="s">
+        <v>12</v>
+      </c>
+      <c r="E28" t="s">
+        <v>13</v>
+      </c>
+      <c r="F28" t="s">
+        <v>149</v>
+      </c>
+      <c r="G28" t="s">
+        <v>150</v>
+      </c>
+      <c r="H28" t="s">
+        <v>16</v>
+      </c>
+      <c r="I28" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="29" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>152</v>
+      </c>
+      <c r="B29" t="s">
+        <v>153</v>
+      </c>
+      <c r="C29" t="s">
+        <v>154</v>
+      </c>
+      <c r="D29" t="s">
+        <v>12</v>
+      </c>
+      <c r="E29" t="s">
+        <v>155</v>
+      </c>
+      <c r="F29" t="s">
+        <v>156</v>
+      </c>
+      <c r="G29" t="s">
+        <v>157</v>
+      </c>
+      <c r="H29" t="s">
+        <v>16</v>
+      </c>
+      <c r="I29" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="30" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>159</v>
+      </c>
+      <c r="B30" t="s">
+        <v>10</v>
+      </c>
+      <c r="C30" t="s">
+        <v>160</v>
+      </c>
+      <c r="D30" t="s">
+        <v>12</v>
+      </c>
+      <c r="E30" t="s">
+        <v>160</v>
+      </c>
+      <c r="F30" t="s">
+        <v>161</v>
+      </c>
+      <c r="G30" t="s">
+        <v>162</v>
+      </c>
+      <c r="H30" t="s">
+        <v>16</v>
+      </c>
+      <c r="I30" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="31" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>164</v>
+      </c>
+      <c r="B31" t="s">
+        <v>10</v>
+      </c>
+      <c r="C31" t="s">
+        <v>165</v>
+      </c>
+      <c r="D31" t="s">
+        <v>12</v>
+      </c>
+      <c r="E31" t="s">
+        <v>13</v>
+      </c>
+      <c r="F31" t="s">
+        <v>166</v>
+      </c>
+      <c r="G31" t="s">
+        <v>167</v>
+      </c>
+      <c r="H31" t="s">
+        <v>16</v>
+      </c>
+      <c r="I31" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="32" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>169</v>
+      </c>
+      <c r="B32" t="s">
+        <v>10</v>
+      </c>
+      <c r="C32" t="s">
+        <v>170</v>
+      </c>
+      <c r="D32" t="s">
+        <v>12</v>
+      </c>
+      <c r="E32" t="s">
+        <v>13</v>
+      </c>
+      <c r="F32" t="s">
+        <v>171</v>
+      </c>
+      <c r="G32" t="s">
+        <v>172</v>
+      </c>
+      <c r="H32" t="s">
+        <v>16</v>
+      </c>
+      <c r="I32" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="33" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>174</v>
+      </c>
+      <c r="B33" t="s">
+        <v>10</v>
+      </c>
+      <c r="C33" t="s">
+        <v>175</v>
+      </c>
+      <c r="D33" t="s">
+        <v>12</v>
+      </c>
+      <c r="E33" t="s">
+        <v>13</v>
+      </c>
+      <c r="F33" t="s">
+        <v>176</v>
+      </c>
+      <c r="G33" t="s">
+        <v>177</v>
+      </c>
+      <c r="H33" t="s">
+        <v>16</v>
+      </c>
+      <c r="I33" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="34" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>179</v>
+      </c>
+      <c r="B34" t="s">
+        <v>10</v>
+      </c>
+      <c r="C34" t="s">
+        <v>180</v>
+      </c>
+      <c r="D34" t="s">
+        <v>12</v>
+      </c>
+      <c r="E34" t="s">
+        <v>13</v>
+      </c>
+      <c r="F34" t="s">
+        <v>181</v>
+      </c>
+      <c r="G34" t="s">
+        <v>182</v>
+      </c>
+      <c r="H34" t="s">
+        <v>16</v>
+      </c>
+      <c r="I34" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="35" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>184</v>
+      </c>
+      <c r="B35" t="s">
+        <v>10</v>
+      </c>
+      <c r="C35" t="s">
+        <v>185</v>
+      </c>
+      <c r="D35" t="s">
+        <v>12</v>
+      </c>
+      <c r="E35" t="s">
+        <v>13</v>
+      </c>
+      <c r="F35" t="s">
+        <v>186</v>
+      </c>
+      <c r="G35" t="s">
+        <v>187</v>
+      </c>
+      <c r="H35" t="s">
+        <v>16</v>
+      </c>
+      <c r="I35" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="36" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>189</v>
+      </c>
+      <c r="B36" t="s">
+        <v>190</v>
+      </c>
+      <c r="C36" t="s">
+        <v>191</v>
+      </c>
+      <c r="D36" t="s">
+        <v>12</v>
+      </c>
+      <c r="E36" t="s">
+        <v>42</v>
+      </c>
+      <c r="F36" t="s">
+        <v>192</v>
+      </c>
+      <c r="G36" t="s">
         <v>21</v>
       </c>
-      <c r="C14" t="s">
-        <v>76</v>
-      </c>
-      <c r="D14" t="s">
-        <v>11</v>
-      </c>
-      <c r="E14" t="s">
-        <v>57</v>
-      </c>
-      <c r="F14" t="s">
-        <v>77</v>
-      </c>
-      <c r="G14" t="s">
-        <v>59</v>
-      </c>
-      <c r="H14" t="s">
-        <v>60</v>
+      <c r="H36" t="s">
+        <v>16</v>
+      </c>
+      <c r="I36" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="37" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>193</v>
+      </c>
+      <c r="B37" t="s">
+        <v>29</v>
+      </c>
+      <c r="C37" t="s">
+        <v>194</v>
+      </c>
+      <c r="D37" t="s">
+        <v>12</v>
+      </c>
+      <c r="E37" t="s">
+        <v>103</v>
+      </c>
+      <c r="F37" t="s">
+        <v>195</v>
+      </c>
+      <c r="G37" t="s">
+        <v>105</v>
+      </c>
+      <c r="H37" t="s">
+        <v>16</v>
+      </c>
+      <c r="I37" t="s">
+        <v>106</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H1"/>
+  <autoFilter ref="A1:I1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>

</xml_diff>